<commit_message>
[tc-night] DSR-529 re-baseline done
</commit_message>
<xml_diff>
--- a/ykk-dsr/hub/tc-out/[Sutrix] DSR -356- [レイアウト] 記事詳細（article-detail）.xlsx
+++ b/ykk-dsr/hub/tc-out/[Sutrix] DSR -356- [レイアウト] 記事詳細（article-detail）.xlsx
@@ -2037,7 +2037,7 @@
       </c>
       <c r="C18" s="95" t="inlineStr">
         <is>
-          <t>EN: Verify the info bar shows publishDate in the design format. JP: 情報バーに掲載日が設計どおりの形式で表示されることを確認する。</t>
+          <t>EN: Verify the info bar shows publishDate as YYYY.MM.DD, the same date as meta publicationdate. JP: 情報バーに掲載日が YYYY.MM.DD 形式で表示され、meta publicationdate と同日であることを確認する。</t>
         </is>
       </c>
       <c r="D18" s="95" t="inlineStr">
@@ -2047,12 +2047,12 @@
       </c>
       <c r="E18" s="95" t="inlineStr">
         <is>
-          <t>EN: 1. Open the page. 2. Read the date text in the info bar. JP: 1. ページを開く。2. 日付表示を確認。</t>
+          <t>EN: 1. Open the page. 2. Read the date text in the info bar. 3. Fetch Publish HTML and read &lt;meta name=publicationdate&gt;. JP: 1. ページを開く。2. 日付表示を確認。3. HTML取得し meta publicationdate を確認。</t>
         </is>
       </c>
       <c r="F18" s="95" t="inlineStr">
         <is>
-          <t>EN: Date text = 2026.10.01 (format YYYY.MM.DD per Figma); same date as meta published-date. JP: 2026.10.01 表示、meta と同日。</t>
+          <t>EN: Date text = 2026.10.01 exactly (YYYY.MM.DD, zero-padded, dot separator) in every language; same date as meta publicationdate. Any other format (2026/10/01, Oct 1, 2026, 2026-10-01, 2026年10月1日) = Fail. JP: 全言語で 2026.10.01（YYYY.MM.DD）表示、meta publicationdate と同日。他形式は Fail。</t>
         </is>
       </c>
       <c r="G18" s="95" t="n"/>
@@ -2074,7 +2074,7 @@
       <c r="K18" s="95" t="n"/>
       <c r="L18" s="96" t="inlineStr">
         <is>
-          <t>Figma #7 (YYYY.MM.DD); property publishDate</t>
+          <t>Figma #7 (YYYY.MM.DD); property publishDate; BUG-RULES §6 (date = YYYY.MM.DD all languages); DSR-660</t>
         </is>
       </c>
       <c r="M18" s="96" t="n"/>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="U18" s="97" t="inlineStr">
         <is>
-          <t>[Giả định] format YYYY.MM.DD for ja/en/cn – Q4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V18" s="59" t="n"/>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="C21" s="95" t="inlineStr">
         <is>
-          <t>EN: Verify meta published-date and updated-date are output in ISO 8601 once each, and updateDate is not displayed on screen. JP: meta published-date／updated-date がISO 8601で1つずつ出力され、更新日は画面に表示されないことを確認する。</t>
+          <t>EN: Verify meta publicationdate and updatedate are output in ISO 8601 once each, and updateDate is not displayed on screen. JP: meta publicationdate／updatedate がISO 8601で1つずつ出力され、更新日は画面に表示されないことを確認する。</t>
         </is>
       </c>
       <c r="D21" s="95" t="inlineStr">
@@ -2329,12 +2329,12 @@
       </c>
       <c r="E21" s="95" t="inlineStr">
         <is>
-          <t>EN: 1. Fetch Publish HTML. 2. Read &lt;meta name=published-date|updated-date&gt;. 3. Search visible text for 2026.10.10 / 2026-10-10. JP: 1. HTML取得。2. meta確認。3. 画面テキスト確認。</t>
+          <t>EN: 1. Fetch Publish HTML. 2. Read &lt;meta name=publicationdate&gt; and &lt;meta name=updatedate&gt; (no hyphen). 3. Search visible text for 2026.10.10 / 2026-10-10. JP: 1. HTML取得。2. meta publicationdate／updatedate 確認（ハイフンなし）。3. 画面テキスト確認。</t>
         </is>
       </c>
       <c r="F21" s="95" t="inlineStr">
         <is>
-          <t>EN: published-date starts with 2026-10-01, updated-date starts with 2026-10-10, both parse as ISO 8601, 1 tag each; update date not visible. JP: ISO 8601、各1件、更新日は非表示。</t>
+          <t>EN: publicationdate starts with 2026-10-01, updatedate starts with 2026-10-10, both parse as ISO 8601, exactly 1 tag each; update date not visible. Hyphenated names (published-date/updated-date) are NOT expected (#58594 outdated). JP: ISO 8601、各1件、更新日は非表示。ハイフン付き名称は旧仕様。</t>
         </is>
       </c>
       <c r="G21" s="95" t="n"/>
@@ -2356,7 +2356,7 @@
       <c r="K21" s="95" t="n"/>
       <c r="L21" s="96" t="inlineStr">
         <is>
-          <t>Property table publishDate/updateDate; Martin §A</t>
+          <t>Property table publishDate/updateDate; Martin §A; re-baseline 2026-10-21 (bugs/529-decision-20261021.md, Martin 21/10)</t>
         </is>
       </c>
       <c r="M21" s="96" t="n"/>
@@ -2507,7 +2507,7 @@
       </c>
       <c r="C23" s="95" t="inlineStr">
         <is>
-          <t>EN: Verify meta category is comma-separated tag IDs and search-keywords is output but not shown in the page body. JP: meta category がタグIDのカンマ区切り、search-keywords が出力され本文には表示されないことを確認する。</t>
+          <t>EN: Verify meta category is comma-separated tag IDs and meta searchkeywords is output but not shown in the page body. JP: meta category がタグIDのカンマ区切り、searchkeywords が出力され本文には表示されないことを確認する。</t>
         </is>
       </c>
       <c r="D23" s="95" t="inlineStr">
@@ -2517,12 +2517,12 @@
       </c>
       <c r="E23" s="95" t="inlineStr">
         <is>
-          <t>EN: 1. Fetch HTML. 2. Read meta category, search-keywords. 3. Search visible text for qa529kw1. JP: 1. HTML取得。2. meta確認。3. 画面検索。</t>
+          <t>EN: 1. Fetch HTML. 2. Read &lt;meta name=category&gt; and &lt;meta name=searchkeywords&gt; (no hyphen). 3. Search visible text for qa529kw1. JP: 1. HTML取得。2. meta category／searchkeywords 確認。3. 画面検索。</t>
         </is>
       </c>
       <c r="F23" s="95" t="inlineStr">
         <is>
-          <t>EN: category = 2 tag IDs (namespace:path) comma-separated; search-keywords contains qa529kw1 and qa529kw2; keywords not visible. JP: タグID2件、キーワード出力・非表示。</t>
+          <t>EN: category = 2 tag IDs (namespace:path) comma-separated (meta present because categories are authored in TD-529-01); searchkeywords contains qa529kw1 and qa529kw2; keywords not visible. Missing category meta while TD-529-01 has no categories authored = data issue, not Fail. JP: タグID2件（カテゴリ設定時のみ出力）、キーワード出力・非表示。</t>
         </is>
       </c>
       <c r="G23" s="95" t="n"/>
@@ -2544,7 +2544,7 @@
       <c r="K23" s="95" t="n"/>
       <c r="L23" s="96" t="inlineStr">
         <is>
-          <t>Property table categories/searchKeywords; Martin §A</t>
+          <t>Property table categories/searchKeywords; Martin §A; re-baseline 2026-10-21 (bugs/529-decision-20261021.md, Martin 21/10)</t>
         </is>
       </c>
       <c r="M23" s="96" t="n"/>
@@ -2710,7 +2710,7 @@
       </c>
       <c r="F25" s="95" t="inlineStr">
         <is>
-          <t>EN: Count = 1 and non-empty for: title, description, og:title, og:description, og:image, published-date, thumbnail, category; og:title/og:description = authored OGP values; og:image absolute URL 200. JP: 各1件・非空、OGP値一致。</t>
+          <t>EN: Count = 1 and non-empty for: title, description, og:title, og:description, og:image, publicationdate, thumbnail, and category (category only counted when categories are authored – TD-529-01 has 2); og:title/og:description = authored OGP values; og:image absolute URL 200. JP: 各1件・非空（category はカテゴリ設定時のみ）、OGP値一致。</t>
         </is>
       </c>
       <c r="G25" s="95" t="n"/>
@@ -2732,7 +2732,7 @@
       <c r="K25" s="95" t="n"/>
       <c r="L25" s="96" t="inlineStr">
         <is>
-          <t>DSR-356 BAC#4; Martin AC#5</t>
+          <t>DSR-356 BAC#4; Martin AC#5; re-baseline 2026-10-21 (bugs/529-decision-20261021.md, Martin 21/10)</t>
         </is>
       </c>
       <c r="M25" s="96" t="n"/>
@@ -3838,7 +3838,7 @@
       </c>
       <c r="F37" s="95" t="inlineStr">
         <is>
-          <t>EN: 200 JSON; row for qa529-01 has navtitle, thumbnail, published-date, updated-date, search-keywords, related-stories (non-empty where set). JP: 200、該当行に6プロパティ。</t>
+          <t>EN: 200 JSON; row for qa529-01 has navtitle, thumbnail, publicationdate, updatedate, searchkeywords, related-stories (non-empty where set). Index is updated only after the page is (re)published. JP: 200、該当行に6プロパティ（再公開後に反映）。</t>
         </is>
       </c>
       <c r="G37" s="98" t="n"/>
@@ -3860,7 +3860,7 @@
       <c r="K37" s="98" t="n"/>
       <c r="L37" s="96" t="inlineStr">
         <is>
-          <t>Martin prereq #1, AC#1</t>
+          <t>Martin prereq #1, AC#1; re-baseline 2026-10-21 (bugs/529-decision-20261021.md, Martin 21/10)</t>
         </is>
       </c>
       <c r="M37" s="96" t="n"/>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="D39" s="95" t="inlineStr">
         <is>
-          <t>EN: TD-529-01 navTitle set. JP: navTitle 設定済み。</t>
+          <t>EN: TD-529-01 navtitle 'QA529 ナビ' set in Universal Editor &gt; Page properties (not Sites &gt; Page Properties), page republished. JP: navtitle を Universal Editor のページプロパティで設定し再公開済み。</t>
         </is>
       </c>
       <c r="E39" s="95" t="inlineStr">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="F39" s="95" t="inlineStr">
         <is>
-          <t>EN: Breadcrumb present; last item = navTitle (not link); earlier items link to ancestors. JP: 最後＝navTitle（リンクなし）。</t>
+          <t>EN: Breadcrumb present; last item text = navtitle 'QA529 ナビ' (en: 'QA529 Nav'), not a link; earlier items link to ancestors. If navtitle is empty, last item = title. JP: 最後＝navtitle（リンクなし）、未設定時は title。</t>
         </is>
       </c>
       <c r="G39" s="98" t="n"/>
@@ -4048,7 +4048,7 @@
       <c r="K39" s="98" t="n"/>
       <c r="L39" s="96" t="inlineStr">
         <is>
-          <t>Figma パンくず; property navTitle; Martin prereq #4</t>
+          <t>Figma パンくず; property navtitle (UE Page properties); Martin prereq #4; DSR-552; re-baseline 2026-10-21 (bugs/529-decision-20261021.md, Martin 21/10)</t>
         </is>
       </c>
       <c r="M39" s="96" t="n"/>
@@ -4081,7 +4081,7 @@
       </c>
       <c r="U39" s="97" t="inlineStr">
         <is>
-          <t>Martin open decision #4 (breadcrumb in scope?) + DSR-552 – Q9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V39" s="59" t="n"/>
@@ -6373,7 +6373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="47" min="1" max="1"/>
@@ -6646,6 +6646,94 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="100" t="inlineStr">
+        <is>
+          <t>A12</t>
+        </is>
+      </c>
+      <c r="B13" s="100" t="inlineStr">
+        <is>
+          <t>Meta names on DEV are publicationdate / updatedate / searchkeywords / category (lowercase, no hyphen). Martin comment #58594 (published-date, updated-date, search-keywords) is outdated. Applies to TC 7, 10, 12, 14, 26.</t>
+        </is>
+      </c>
+      <c r="C13" s="100" t="inlineStr">
+        <is>
+          <t>Martin 21/10 via Dat; bugs/529-decision-20261021.md (BUG-2 = not a bug)</t>
+        </is>
+      </c>
+      <c r="D13" s="100" t="inlineStr">
+        <is>
+          <t>Re-baseline if dev renames again</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="100" t="inlineStr">
+        <is>
+          <t>A13</t>
+        </is>
+      </c>
+      <c r="B14" s="100" t="inlineStr">
+        <is>
+          <t>meta category is output only when at least 1 category is authored; absence with no categories = expected, not Fail.</t>
+        </is>
+      </c>
+      <c r="C14" s="100" t="inlineStr">
+        <is>
+          <t>Martin 21/10; bugs/529-decision-20261021.md</t>
+        </is>
+      </c>
+      <c r="D14" s="100" t="inlineStr">
+        <is>
+          <t>TC 12, 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="100" t="inlineStr">
+        <is>
+          <t>A14</t>
+        </is>
+      </c>
+      <c r="B15" s="100" t="inlineStr">
+        <is>
+          <t>navtitle (Navigation Title) is authored in Universal Editor &gt; Page properties, not in Sites &gt; Page Properties; it is the last breadcrumb item. Index/meta update only after republish.</t>
+        </is>
+      </c>
+      <c r="C15" s="100" t="inlineStr">
+        <is>
+          <t>Martin 21/10; bugs/529-decision-20261021.md (NEW-1 = not a bug)</t>
+        </is>
+      </c>
+      <c r="D15" s="100" t="inlineStr">
+        <is>
+          <t>TC 26, 28; TD-529-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="100" t="inlineStr">
+        <is>
+          <t>A15</t>
+        </is>
+      </c>
+      <c r="B16" s="100" t="inlineStr">
+        <is>
+          <t>Date display = YYYY.MM.DD in every language (ja/en/cn); replaces the Q4 assumption.</t>
+        </is>
+      </c>
+      <c r="C16" s="100" t="inlineStr">
+        <is>
+          <t>BUG-RULES §6; DSR-660</t>
+        </is>
+      </c>
+      <c r="D16" s="100" t="inlineStr">
+        <is>
+          <t>TC 7, 18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>